<commit_message>
Marketing kit: trim Google Ads copy to limits, refresh spreadsheets and zip
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y2F4PbSnsXwQDZgW2qnbaK
</commit_message>
<xml_diff>
--- a/marketing-kit/advertising/ad-copy-bank.xlsx
+++ b/marketing-kit/advertising/ad-copy-bank.xlsx
@@ -930,7 +930,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Monthly Lease. No Contract Lock-In</t>
+          <t>Monthly Lease, No Lock-In</t>
         </is>
       </c>
       <c r="C18" s="5">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Add 24/7 professional monitoring for the whole site for $150/mo. Agents warn intruders &amp; call it in.</t>
+          <t>Add 24/7 site monitoring for $150/mo. Live agents warn intruders and call it in.</t>
         </is>
       </c>
       <c r="C21" s="4">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>No power, internet, or trenching needed. Solar + battery + built-in LTE. Live the day it arrives.</t>
+          <t>No power, internet, or trenching needed. Solar + battery + LTE. Live the day it arrives.</t>
         </is>
       </c>
       <c r="C22" s="5">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>12 ft mast, dual 4K cameras, floodlight &amp; siren. Plain-English alerts to your phone. Book a site walk.</t>
+          <t>12 ft mast, dual 4K cameras, floodlight &amp; siren. Plain-English alerts to your phone.</t>
         </is>
       </c>
       <c r="C23" s="4">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Protect copper, tools, lumber &amp; equipment between shifts. Monthly lease that moves with your project.</t>
+          <t>Protect copper, tools &amp; equipment between shifts. Monthly lease moves with your project.</t>
         </is>
       </c>
       <c r="C24" s="5">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Serving Houston, Katy, Sugar Land, The Woodlands, Pearland &amp; beyond. Free consultation, no obligation.</t>
+          <t>Serving Houston, Katy, Sugar Land, The Woodlands &amp; Pearland. Free consultation.</t>
         </is>
       </c>
       <c r="C25" s="4">

</xml_diff>